<commit_message>
Add automatic market data update for portfolio Excel
- portfolio_fetcher.py: fetch ETF/stock/index quotes via akshare
- update_portfolio_excel.py: update prices across all sheets + log
- run_daily_update.sh/.bat for scheduled updates
- README with setup and cron instructions

Co-authored-by: binenyuan <binenyuan@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/持仓跟踪表_434050.xlsx
+++ b/持仓跟踪表_434050.xlsx
@@ -1,18 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="当前持仓" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="稳健版目标持仓" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="激进版目标持仓" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="每日监控" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="情景压力测试" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="使用说明" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="当前持仓" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="稳健版目标持仓" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="激进版目标持仓" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="每日监控" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="情景压力测试" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使用说明" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据更新日志" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -22,8 +23,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
   <fonts count="5">
     <font>
@@ -82,7 +83,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -95,10 +96,10 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -120,10 +121,21 @@
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -518,11 +530,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>基准日期：2026-07-17  |  账户总市值：</t>
-        </is>
-      </c>
-      <c r="K2" s="2" t="n">
-        <v>434050</v>
+          <t>数据更新：2026-07-19 06:52  |  行情日期：2026-07-19  |  账户总市值：</t>
+        </is>
+      </c>
+      <c r="K2" s="2">
+        <f>SUM(G5:G15)</f>
+        <v/>
       </c>
       <c r="L2" t="inlineStr">
         <is>
@@ -619,17 +632,17 @@
       <c r="D5" s="5" t="n">
         <v>26100</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="19" t="n">
         <v>1.905</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="19" t="n">
         <v>2.557</v>
       </c>
       <c r="G5" s="5">
         <f>D5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="7">
+      <c r="H5" s="20">
         <f>G5/$K$2</f>
         <v/>
       </c>
@@ -637,7 +650,7 @@
         <f>(F5-E5)*D5</f>
         <v/>
       </c>
-      <c r="J5" s="7">
+      <c r="J5" s="20">
         <f>IF(E5=0,0,(F5-E5)/E5)</f>
         <v/>
       </c>
@@ -673,17 +686,17 @@
       <c r="D6" s="5" t="n">
         <v>32500</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="19" t="n">
         <v>1.82</v>
       </c>
       <c r="G6" s="5">
         <f>D6*F6</f>
         <v/>
       </c>
-      <c r="H6" s="7">
+      <c r="H6" s="20">
         <f>G6/$K$2</f>
         <v/>
       </c>
@@ -691,7 +704,7 @@
         <f>(F6-E6)*D6</f>
         <v/>
       </c>
-      <c r="J6" s="7">
+      <c r="J6" s="20">
         <f>IF(E6=0,0,(F6-E6)/E6)</f>
         <v/>
       </c>
@@ -727,17 +740,17 @@
       <c r="D7" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="19" t="n">
         <v>249.537</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="19" t="n">
         <v>241.92</v>
       </c>
       <c r="G7" s="5">
         <f>D7*F7</f>
         <v/>
       </c>
-      <c r="H7" s="7">
+      <c r="H7" s="20">
         <f>G7/$K$2</f>
         <v/>
       </c>
@@ -745,7 +758,7 @@
         <f>(F7-E7)*D7</f>
         <v/>
       </c>
-      <c r="J7" s="7">
+      <c r="J7" s="20">
         <f>IF(E7=0,0,(F7-E7)/E7)</f>
         <v/>
       </c>
@@ -781,17 +794,17 @@
       <c r="D8" s="5" t="n">
         <v>800</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="19" t="n">
         <v>69.398</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="19" t="n">
         <v>58.05</v>
       </c>
       <c r="G8" s="5">
         <f>D8*F8</f>
         <v/>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="20">
         <f>G8/$K$2</f>
         <v/>
       </c>
@@ -799,7 +812,7 @@
         <f>(F8-E8)*D8</f>
         <v/>
       </c>
-      <c r="J8" s="7">
+      <c r="J8" s="20">
         <f>IF(E8=0,0,(F8-E8)/E8)</f>
         <v/>
       </c>
@@ -835,17 +848,17 @@
       <c r="D9" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E9" s="19" t="n">
         <v>79.88200000000001</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="19" t="n">
         <v>71.7</v>
       </c>
       <c r="G9" s="5">
         <f>D9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="20">
         <f>G9/$K$2</f>
         <v/>
       </c>
@@ -853,7 +866,7 @@
         <f>(F9-E9)*D9</f>
         <v/>
       </c>
-      <c r="J9" s="7">
+      <c r="J9" s="20">
         <f>IF(E9=0,0,(F9-E9)/E9)</f>
         <v/>
       </c>
@@ -889,17 +902,17 @@
       <c r="D10" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="19" t="n">
         <v>185.479</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="19" t="n">
         <v>132.29</v>
       </c>
       <c r="G10" s="5">
         <f>D10*F10</f>
         <v/>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="20">
         <f>G10/$K$2</f>
         <v/>
       </c>
@@ -907,7 +920,7 @@
         <f>(F10-E10)*D10</f>
         <v/>
       </c>
-      <c r="J10" s="7">
+      <c r="J10" s="20">
         <f>IF(E10=0,0,(F10-E10)/E10)</f>
         <v/>
       </c>
@@ -943,17 +956,17 @@
       <c r="D11" s="5" t="n">
         <v>59700</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="19" t="n">
         <v>0.506</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="19" t="n">
         <v>0.659</v>
       </c>
       <c r="G11" s="5">
         <f>D11*F11</f>
         <v/>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="20">
         <f>G11/$K$2</f>
         <v/>
       </c>
@@ -961,7 +974,7 @@
         <f>(F11-E11)*D11</f>
         <v/>
       </c>
-      <c r="J11" s="7">
+      <c r="J11" s="20">
         <f>IF(E11=0,0,(F11-E11)/E11)</f>
         <v/>
       </c>
@@ -997,17 +1010,17 @@
       <c r="D12" s="5" t="n">
         <v>500</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="19" t="n">
         <v>109.457</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="19" t="n">
         <v>58.39</v>
       </c>
       <c r="G12" s="5">
         <f>D12*F12</f>
         <v/>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="20">
         <f>G12/$K$2</f>
         <v/>
       </c>
@@ -1015,7 +1028,7 @@
         <f>(F12-E12)*D12</f>
         <v/>
       </c>
-      <c r="J12" s="7">
+      <c r="J12" s="20">
         <f>IF(E12=0,0,(F12-E12)/E12)</f>
         <v/>
       </c>
@@ -1047,17 +1060,17 @@
       <c r="D13" s="5" t="n">
         <v>300</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="19" t="n">
         <v>128.923</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="19" t="n">
         <v>96.19</v>
       </c>
       <c r="G13" s="5">
         <f>D13*F13</f>
         <v/>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="20">
         <f>G13/$K$2</f>
         <v/>
       </c>
@@ -1065,7 +1078,7 @@
         <f>(F13-E13)*D13</f>
         <v/>
       </c>
-      <c r="J13" s="7">
+      <c r="J13" s="20">
         <f>IF(E13=0,0,(F13-E13)/E13)</f>
         <v/>
       </c>
@@ -1097,17 +1110,17 @@
       <c r="D14" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="19" t="n">
         <v>78.211</v>
       </c>
-      <c r="F14" s="6" t="n">
+      <c r="F14" s="19" t="n">
         <v>68.36</v>
       </c>
       <c r="G14" s="5">
         <f>D14*F14</f>
         <v/>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="20">
         <f>G14/$K$2</f>
         <v/>
       </c>
@@ -1115,7 +1128,7 @@
         <f>(F14-E14)*D14</f>
         <v/>
       </c>
-      <c r="J14" s="7">
+      <c r="J14" s="20">
         <f>IF(E14=0,0,(F14-E14)/E14)</f>
         <v/>
       </c>
@@ -1151,17 +1164,17 @@
       <c r="D15" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E15" s="19" t="n">
         <v>76.93000000000001</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="19" t="n">
         <v>60.05</v>
       </c>
       <c r="G15" s="5">
         <f>D15*F15</f>
         <v/>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="20">
         <f>G15/$K$2</f>
         <v/>
       </c>
@@ -1169,7 +1182,7 @@
         <f>(F15-E15)*D15</f>
         <v/>
       </c>
-      <c r="J15" s="7">
+      <c r="J15" s="20">
         <f>IF(E15=0,0,(F15-E15)/E15)</f>
         <v/>
       </c>
@@ -1203,7 +1216,7 @@
         <f>SUM(G5:G15)</f>
         <v/>
       </c>
-      <c r="H16" s="7">
+      <c r="H16" s="20">
         <f>SUM(H5:H15)</f>
         <v/>
       </c>
@@ -1211,7 +1224,7 @@
         <f>SUM(I5:I15)</f>
         <v/>
       </c>
-      <c r="J16" s="7">
+      <c r="J16" s="20">
         <f>IF(G16-I16=0,0,I16/(G16-I16))</f>
         <v/>
       </c>
@@ -1372,20 +1385,20 @@
       <c r="D5" s="5" t="n">
         <v>14355</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="19" t="n">
         <v>1.905</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="19" t="n">
         <v>2.557</v>
       </c>
       <c r="G5" s="5">
         <f>D5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="20" t="n">
         <v>0.08500000000000001</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="20">
         <f>G5/$B$2</f>
         <v/>
       </c>
@@ -1393,7 +1406,7 @@
         <f>(F5-E5)*D5</f>
         <v/>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="20">
         <f>IF(E5=0,0,(F5-E5)/E5)</f>
         <v/>
       </c>
@@ -1403,7 +1416,7 @@
       <c r="M5" s="9" t="n">
         <v>2.8</v>
       </c>
-      <c r="N5" s="7">
+      <c r="N5" s="20">
         <f>IF(L5="","",(F5-L5)/L5)</f>
         <v/>
       </c>
@@ -1434,20 +1447,20 @@
       <c r="D6" s="5" t="n">
         <v>16250</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="19" t="n">
         <v>1.82</v>
       </c>
       <c r="G6" s="5">
         <f>D6*F6</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="20" t="n">
         <v>0.068</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="20">
         <f>G6/$B$2</f>
         <v/>
       </c>
@@ -1455,7 +1468,7 @@
         <f>(F6-E6)*D6</f>
         <v/>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="20">
         <f>IF(E6=0,0,(F6-E6)/E6)</f>
         <v/>
       </c>
@@ -1465,7 +1478,7 @@
       <c r="M6" s="9" t="n">
         <v>1.95</v>
       </c>
-      <c r="N6" s="7">
+      <c r="N6" s="20">
         <f>IF(L6="","",(F6-L6)/L6)</f>
         <v/>
       </c>
@@ -1496,20 +1509,20 @@
       <c r="D7" s="5" t="n">
         <v>26865</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.506</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.659</v>
       </c>
       <c r="G7" s="5">
         <f>D7*F7</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="20" t="n">
         <v>0.041</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="20">
         <f>G7/$B$2</f>
         <v/>
       </c>
@@ -1517,7 +1530,7 @@
         <f>(F7-E7)*D7</f>
         <v/>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="20">
         <f>IF(E7=0,0,(F7-E7)/E7)</f>
         <v/>
       </c>
@@ -1527,7 +1540,7 @@
       <c r="M7" s="9" t="n">
         <v>0.72</v>
       </c>
-      <c r="N7" s="7">
+      <c r="N7" s="20">
         <f>IF(L7="","",(F7-L7)/L7)</f>
         <v/>
       </c>
@@ -1558,20 +1571,20 @@
       <c r="D8" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="19" t="n">
         <v>79.88200000000001</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="19" t="n">
         <v>71.7</v>
       </c>
       <c r="G8" s="5">
         <f>D8*F8</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="20" t="n">
         <v>0.099</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="20">
         <f>G8/$B$2</f>
         <v/>
       </c>
@@ -1579,7 +1592,7 @@
         <f>(F8-E8)*D8</f>
         <v/>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="20">
         <f>IF(E8=0,0,(F8-E8)/E8)</f>
         <v/>
       </c>
@@ -1589,7 +1602,7 @@
       <c r="M8" s="9" t="n">
         <v>80</v>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="20">
         <f>IF(L8="","",(F8-L8)/L8)</f>
         <v/>
       </c>
@@ -1620,20 +1633,20 @@
       <c r="D9" s="5" t="n">
         <v>800</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E9" s="19" t="n">
         <v>69.398</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="19" t="n">
         <v>58.05</v>
       </c>
       <c r="G9" s="5">
         <f>D9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="20" t="n">
         <v>0.107</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="20">
         <f>G9/$B$2</f>
         <v/>
       </c>
@@ -1641,7 +1654,7 @@
         <f>(F9-E9)*D9</f>
         <v/>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="20">
         <f>IF(E9=0,0,(F9-E9)/E9)</f>
         <v/>
       </c>
@@ -1651,7 +1664,7 @@
       <c r="M9" s="9" t="n">
         <v>68</v>
       </c>
-      <c r="N9" s="7">
+      <c r="N9" s="20">
         <f>IF(L9="","",(F9-L9)/L9)</f>
         <v/>
       </c>
@@ -1682,20 +1695,20 @@
       <c r="D10" s="5" t="n">
         <v>100</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="19" t="n">
         <v>249.537</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="19" t="n">
         <v>241.92</v>
       </c>
       <c r="G10" s="5">
         <f>D10*F10</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="20" t="n">
         <v>0.056</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="20">
         <f>G10/$B$2</f>
         <v/>
       </c>
@@ -1703,7 +1716,7 @@
         <f>(F10-E10)*D10</f>
         <v/>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="20">
         <f>IF(E10=0,0,(F10-E10)/E10)</f>
         <v/>
       </c>
@@ -1713,7 +1726,7 @@
       <c r="M10" s="9" t="n">
         <v>260</v>
       </c>
-      <c r="N10" s="7">
+      <c r="N10" s="20">
         <f>IF(L10="","",(F10-L10)/L10)</f>
         <v/>
       </c>
@@ -1744,20 +1757,20 @@
       <c r="D11" s="5" t="n">
         <v>16500</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="19" t="n">
         <v>3.15</v>
       </c>
-      <c r="F11" s="6" t="n">
-        <v>3.15</v>
+      <c r="F11" s="19" t="n">
+        <v>3.135</v>
       </c>
       <c r="G11" s="5">
         <f>D11*F11</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="20" t="n">
         <v>0.12</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="20">
         <f>G11/$B$2</f>
         <v/>
       </c>
@@ -1765,7 +1778,7 @@
         <f>(F11-E11)*D11</f>
         <v/>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="20">
         <f>IF(E11=0,0,(F11-E11)/E11)</f>
         <v/>
       </c>
@@ -1775,7 +1788,7 @@
       <c r="M11" s="9" t="n">
         <v>3.5</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="20">
         <f>IF(L11="","",(F11-L11)/L11)</f>
         <v/>
       </c>
@@ -1806,20 +1819,20 @@
       <c r="D12" s="5" t="n">
         <v>10750</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="F12" s="6" t="n">
-        <v>4</v>
+      <c r="F12" s="19" t="n">
+        <v>4.589</v>
       </c>
       <c r="G12" s="5">
         <f>D12*F12</f>
         <v/>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="20" t="n">
         <v>0.099</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="20">
         <f>G12/$B$2</f>
         <v/>
       </c>
@@ -1827,7 +1840,7 @@
         <f>(F12-E12)*D12</f>
         <v/>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="20">
         <f>IF(E12=0,0,(F12-E12)/E12)</f>
         <v/>
       </c>
@@ -1837,7 +1850,7 @@
       <c r="M12" s="9" t="n">
         <v>4.4</v>
       </c>
-      <c r="N12" s="7">
+      <c r="N12" s="20">
         <f>IF(L12="","",(F12-L12)/L12)</f>
         <v/>
       </c>
@@ -1868,26 +1881,26 @@
       <c r="D13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F13" s="6" t="n">
+      <c r="F13" s="19" t="n">
         <v>1</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>122525</v>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H13" s="20" t="n">
         <v>0.282</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="20">
         <f>G13/$B$2</f>
         <v/>
       </c>
       <c r="J13" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="7" t="n">
+      <c r="K13" s="20" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="10" t="inlineStr"/>
@@ -1924,7 +1937,7 @@
         <v/>
       </c>
       <c r="H14" s="10" t="n"/>
-      <c r="I14" s="7">
+      <c r="I14" s="20">
         <f>SUM(I5:I13)</f>
         <v/>
       </c>
@@ -2500,20 +2513,20 @@
       <c r="D5" s="5" t="n">
         <v>20880</v>
       </c>
-      <c r="E5" s="6" t="n">
+      <c r="E5" s="19" t="n">
         <v>1.905</v>
       </c>
-      <c r="F5" s="6" t="n">
+      <c r="F5" s="19" t="n">
         <v>2.557</v>
       </c>
       <c r="G5" s="5">
         <f>D5*F5</f>
         <v/>
       </c>
-      <c r="H5" s="7" t="n">
+      <c r="H5" s="20" t="n">
         <v>0.123</v>
       </c>
-      <c r="I5" s="7">
+      <c r="I5" s="20">
         <f>G5/$B$2</f>
         <v/>
       </c>
@@ -2521,7 +2534,7 @@
         <f>(F5-E5)*D5</f>
         <v/>
       </c>
-      <c r="K5" s="7">
+      <c r="K5" s="20">
         <f>IF(E5=0,0,(F5-E5)/E5)</f>
         <v/>
       </c>
@@ -2531,7 +2544,7 @@
       <c r="M5" s="10" t="n">
         <v>2.9</v>
       </c>
-      <c r="N5" s="7">
+      <c r="N5" s="20">
         <f>IF(L5="","",(F5-L5)/L5)</f>
         <v/>
       </c>
@@ -2562,20 +2575,20 @@
       <c r="D6" s="5" t="n">
         <v>27625</v>
       </c>
-      <c r="E6" s="6" t="n">
+      <c r="E6" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F6" s="6" t="n">
+      <c r="F6" s="19" t="n">
         <v>1.82</v>
       </c>
       <c r="G6" s="5">
         <f>D6*F6</f>
         <v/>
       </c>
-      <c r="H6" s="7" t="n">
+      <c r="H6" s="20" t="n">
         <v>0.116</v>
       </c>
-      <c r="I6" s="7">
+      <c r="I6" s="20">
         <f>G6/$B$2</f>
         <v/>
       </c>
@@ -2583,7 +2596,7 @@
         <f>(F6-E6)*D6</f>
         <v/>
       </c>
-      <c r="K6" s="7">
+      <c r="K6" s="20">
         <f>IF(E6=0,0,(F6-E6)/E6)</f>
         <v/>
       </c>
@@ -2593,7 +2606,7 @@
       <c r="M6" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="N6" s="7">
+      <c r="N6" s="20">
         <f>IF(L6="","",(F6-L6)/L6)</f>
         <v/>
       </c>
@@ -2624,20 +2637,20 @@
       <c r="D7" s="5" t="n">
         <v>44775</v>
       </c>
-      <c r="E7" s="6" t="n">
+      <c r="E7" s="19" t="n">
         <v>0.506</v>
       </c>
-      <c r="F7" s="6" t="n">
+      <c r="F7" s="19" t="n">
         <v>0.659</v>
       </c>
       <c r="G7" s="5">
         <f>D7*F7</f>
         <v/>
       </c>
-      <c r="H7" s="7" t="n">
+      <c r="H7" s="20" t="n">
         <v>0.068</v>
       </c>
-      <c r="I7" s="7">
+      <c r="I7" s="20">
         <f>G7/$B$2</f>
         <v/>
       </c>
@@ -2645,7 +2658,7 @@
         <f>(F7-E7)*D7</f>
         <v/>
       </c>
-      <c r="K7" s="7">
+      <c r="K7" s="20">
         <f>IF(E7=0,0,(F7-E7)/E7)</f>
         <v/>
       </c>
@@ -2655,7 +2668,7 @@
       <c r="M7" s="10" t="n">
         <v>0.75</v>
       </c>
-      <c r="N7" s="7">
+      <c r="N7" s="20">
         <f>IF(L7="","",(F7-L7)/L7)</f>
         <v/>
       </c>
@@ -2686,20 +2699,20 @@
       <c r="D8" s="5" t="n">
         <v>600</v>
       </c>
-      <c r="E8" s="6" t="n">
+      <c r="E8" s="19" t="n">
         <v>79.88200000000001</v>
       </c>
-      <c r="F8" s="6" t="n">
+      <c r="F8" s="19" t="n">
         <v>71.7</v>
       </c>
       <c r="G8" s="5">
         <f>D8*F8</f>
         <v/>
       </c>
-      <c r="H8" s="7" t="n">
+      <c r="H8" s="20" t="n">
         <v>0.099</v>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="20">
         <f>G8/$B$2</f>
         <v/>
       </c>
@@ -2707,7 +2720,7 @@
         <f>(F8-E8)*D8</f>
         <v/>
       </c>
-      <c r="K8" s="7">
+      <c r="K8" s="20">
         <f>IF(E8=0,0,(F8-E8)/E8)</f>
         <v/>
       </c>
@@ -2717,7 +2730,7 @@
       <c r="M8" s="10" t="n">
         <v>85</v>
       </c>
-      <c r="N8" s="7">
+      <c r="N8" s="20">
         <f>IF(L8="","",(F8-L8)/L8)</f>
         <v/>
       </c>
@@ -2748,20 +2761,20 @@
       <c r="D9" s="5" t="n">
         <v>200</v>
       </c>
-      <c r="E9" s="6" t="n">
+      <c r="E9" s="19" t="n">
         <v>249.537</v>
       </c>
-      <c r="F9" s="6" t="n">
+      <c r="F9" s="19" t="n">
         <v>241.92</v>
       </c>
       <c r="G9" s="5">
         <f>D9*F9</f>
         <v/>
       </c>
-      <c r="H9" s="7" t="n">
+      <c r="H9" s="20" t="n">
         <v>0.112</v>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="20">
         <f>G9/$B$2</f>
         <v/>
       </c>
@@ -2769,7 +2782,7 @@
         <f>(F9-E9)*D9</f>
         <v/>
       </c>
-      <c r="K9" s="7">
+      <c r="K9" s="20">
         <f>IF(E9=0,0,(F9-E9)/E9)</f>
         <v/>
       </c>
@@ -2779,7 +2792,7 @@
       <c r="M9" s="10" t="n">
         <v>270</v>
       </c>
-      <c r="N9" s="7">
+      <c r="N9" s="20">
         <f>IF(L9="","",(F9-L9)/L9)</f>
         <v/>
       </c>
@@ -2810,20 +2823,20 @@
       <c r="D10" s="5" t="n">
         <v>800</v>
       </c>
-      <c r="E10" s="6" t="n">
+      <c r="E10" s="19" t="n">
         <v>69.398</v>
       </c>
-      <c r="F10" s="6" t="n">
+      <c r="F10" s="19" t="n">
         <v>58.05</v>
       </c>
       <c r="G10" s="5">
         <f>D10*F10</f>
         <v/>
       </c>
-      <c r="H10" s="7" t="n">
+      <c r="H10" s="20" t="n">
         <v>0.107</v>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="20">
         <f>G10/$B$2</f>
         <v/>
       </c>
@@ -2831,7 +2844,7 @@
         <f>(F10-E10)*D10</f>
         <v/>
       </c>
-      <c r="K10" s="7">
+      <c r="K10" s="20">
         <f>IF(E10=0,0,(F10-E10)/E10)</f>
         <v/>
       </c>
@@ -2841,7 +2854,7 @@
       <c r="M10" s="10" t="n">
         <v>72</v>
       </c>
-      <c r="N10" s="7">
+      <c r="N10" s="20">
         <f>IF(L10="","",(F10-L10)/L10)</f>
         <v/>
       </c>
@@ -2872,20 +2885,20 @@
       <c r="D11" s="5" t="n">
         <v>400</v>
       </c>
-      <c r="E11" s="6" t="n">
+      <c r="E11" s="19" t="n">
         <v>78.211</v>
       </c>
-      <c r="F11" s="6" t="n">
+      <c r="F11" s="19" t="n">
         <v>68.36</v>
       </c>
       <c r="G11" s="5">
         <f>D11*F11</f>
         <v/>
       </c>
-      <c r="H11" s="7" t="n">
+      <c r="H11" s="20" t="n">
         <v>0.063</v>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="20">
         <f>G11/$B$2</f>
         <v/>
       </c>
@@ -2893,7 +2906,7 @@
         <f>(F11-E11)*D11</f>
         <v/>
       </c>
-      <c r="K11" s="7">
+      <c r="K11" s="20">
         <f>IF(E11=0,0,(F11-E11)/E11)</f>
         <v/>
       </c>
@@ -2903,7 +2916,7 @@
       <c r="M11" s="10" t="n">
         <v>82</v>
       </c>
-      <c r="N11" s="7">
+      <c r="N11" s="20">
         <f>IF(L11="","",(F11-L11)/L11)</f>
         <v/>
       </c>
@@ -2934,20 +2947,20 @@
       <c r="D12" s="5" t="n">
         <v>150</v>
       </c>
-      <c r="E12" s="6" t="n">
+      <c r="E12" s="19" t="n">
         <v>185.479</v>
       </c>
-      <c r="F12" s="6" t="n">
+      <c r="F12" s="19" t="n">
         <v>132.29</v>
       </c>
       <c r="G12" s="5">
         <f>D12*F12</f>
         <v/>
       </c>
-      <c r="H12" s="7" t="n">
+      <c r="H12" s="20" t="n">
         <v>0.046</v>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="20">
         <f>G12/$B$2</f>
         <v/>
       </c>
@@ -2955,7 +2968,7 @@
         <f>(F12-E12)*D12</f>
         <v/>
       </c>
-      <c r="K12" s="7">
+      <c r="K12" s="20">
         <f>IF(E12=0,0,(F12-E12)/E12)</f>
         <v/>
       </c>
@@ -2965,7 +2978,7 @@
       <c r="M12" s="10" t="n">
         <v>160</v>
       </c>
-      <c r="N12" s="7">
+      <c r="N12" s="20">
         <f>IF(L12="","",(F12-L12)/L12)</f>
         <v/>
       </c>
@@ -2996,20 +3009,20 @@
       <c r="D13" s="5" t="n">
         <v>7000</v>
       </c>
-      <c r="E13" s="6" t="n">
+      <c r="E13" s="19" t="n">
         <v>3.15</v>
       </c>
-      <c r="F13" s="6" t="n">
-        <v>3.15</v>
+      <c r="F13" s="19" t="n">
+        <v>3.135</v>
       </c>
       <c r="G13" s="5">
         <f>D13*F13</f>
         <v/>
       </c>
-      <c r="H13" s="7" t="n">
+      <c r="H13" s="20" t="n">
         <v>0.051</v>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="20">
         <f>G13/$B$2</f>
         <v/>
       </c>
@@ -3017,7 +3030,7 @@
         <f>(F13-E13)*D13</f>
         <v/>
       </c>
-      <c r="K13" s="7">
+      <c r="K13" s="20">
         <f>IF(E13=0,0,(F13-E13)/E13)</f>
         <v/>
       </c>
@@ -3027,7 +3040,7 @@
       <c r="M13" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="N13" s="7">
+      <c r="N13" s="20">
         <f>IF(L13="","",(F13-L13)/L13)</f>
         <v/>
       </c>
@@ -3058,20 +3071,20 @@
       <c r="D14" s="5" t="n">
         <v>3250</v>
       </c>
-      <c r="E14" s="6" t="n">
+      <c r="E14" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="F14" s="6" t="n">
-        <v>4</v>
+      <c r="F14" s="19" t="n">
+        <v>4.589</v>
       </c>
       <c r="G14" s="5">
         <f>D14*F14</f>
         <v/>
       </c>
-      <c r="H14" s="7" t="n">
+      <c r="H14" s="20" t="n">
         <v>0.03</v>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="20">
         <f>G14/$B$2</f>
         <v/>
       </c>
@@ -3079,7 +3092,7 @@
         <f>(F14-E14)*D14</f>
         <v/>
       </c>
-      <c r="K14" s="7">
+      <c r="K14" s="20">
         <f>IF(E14=0,0,(F14-E14)/E14)</f>
         <v/>
       </c>
@@ -3089,7 +3102,7 @@
       <c r="M14" s="10" t="n">
         <v>4.4</v>
       </c>
-      <c r="N14" s="7">
+      <c r="N14" s="20">
         <f>IF(L14="","",(F14-L14)/L14)</f>
         <v/>
       </c>
@@ -3120,26 +3133,26 @@
       <c r="D15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="6" t="n">
+      <c r="E15" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F15" s="6" t="n">
+      <c r="F15" s="19" t="n">
         <v>1</v>
       </c>
       <c r="G15" s="5" t="n">
         <v>80956</v>
       </c>
-      <c r="H15" s="7" t="n">
+      <c r="H15" s="20" t="n">
         <v>0.187</v>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="20">
         <f>G15/$B$2</f>
         <v/>
       </c>
       <c r="J15" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="7" t="n">
+      <c r="K15" s="20" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="10" t="inlineStr"/>
@@ -3176,7 +3189,7 @@
         <v/>
       </c>
       <c r="H16" s="10" t="n"/>
-      <c r="I16" s="7">
+      <c r="I16" s="20">
         <f>SUM(I5:I15)</f>
         <v/>
       </c>
@@ -3592,7 +3605,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-19 06:52</t>
         </is>
       </c>
     </row>
@@ -3602,8 +3615,8 @@
           <t>沪指收盘：</t>
         </is>
       </c>
-      <c r="B4" t="n">
-        <v>3764.15</v>
+      <c r="B4" s="21" t="n">
+        <v>3764.155</v>
       </c>
     </row>
     <row r="5">
@@ -3699,11 +3712,11 @@
       <c r="G8" s="10" t="n">
         <v>2.8</v>
       </c>
-      <c r="H8" s="7">
+      <c r="H8" s="20">
         <f>IF(F8=0,"",(E8-F8)/F8)</f>
         <v/>
       </c>
-      <c r="I8" s="7">
+      <c r="I8" s="20">
         <f>IF(G8=0,"",(G8-E8)/E8)</f>
         <v/>
       </c>
@@ -3742,11 +3755,11 @@
       <c r="G9" s="10" t="n">
         <v>1.95</v>
       </c>
-      <c r="H9" s="7">
+      <c r="H9" s="20">
         <f>IF(F9=0,"",(E9-F9)/F9)</f>
         <v/>
       </c>
-      <c r="I9" s="7">
+      <c r="I9" s="20">
         <f>IF(G9=0,"",(G9-E9)/E9)</f>
         <v/>
       </c>
@@ -3785,11 +3798,11 @@
       <c r="G10" s="10" t="n">
         <v>0.72</v>
       </c>
-      <c r="H10" s="7">
+      <c r="H10" s="20">
         <f>IF(F10=0,"",(E10-F10)/F10)</f>
         <v/>
       </c>
-      <c r="I10" s="7">
+      <c r="I10" s="20">
         <f>IF(G10=0,"",(G10-E10)/E10)</f>
         <v/>
       </c>
@@ -3828,11 +3841,11 @@
       <c r="G11" s="10" t="n">
         <v>80</v>
       </c>
-      <c r="H11" s="7">
+      <c r="H11" s="20">
         <f>IF(F11=0,"",(E11-F11)/F11)</f>
         <v/>
       </c>
-      <c r="I11" s="7">
+      <c r="I11" s="20">
         <f>IF(G11=0,"",(G11-E11)/E11)</f>
         <v/>
       </c>
@@ -3871,11 +3884,11 @@
       <c r="G12" s="10" t="n">
         <v>68</v>
       </c>
-      <c r="H12" s="7">
+      <c r="H12" s="20">
         <f>IF(F12=0,"",(E12-F12)/F12)</f>
         <v/>
       </c>
-      <c r="I12" s="7">
+      <c r="I12" s="20">
         <f>IF(G12=0,"",(G12-E12)/E12)</f>
         <v/>
       </c>
@@ -3914,11 +3927,11 @@
       <c r="G13" s="10" t="n">
         <v>260</v>
       </c>
-      <c r="H13" s="7">
+      <c r="H13" s="20">
         <f>IF(F13=0,"",(E13-F13)/F13)</f>
         <v/>
       </c>
-      <c r="I13" s="7">
+      <c r="I13" s="20">
         <f>IF(G13=0,"",(G13-E13)/E13)</f>
         <v/>
       </c>
@@ -3949,7 +3962,7 @@
         <v>3.15</v>
       </c>
       <c r="E14" s="10" t="n">
-        <v>3.15</v>
+        <v>3.135</v>
       </c>
       <c r="F14" s="10" t="n">
         <v>2.9</v>
@@ -3957,11 +3970,11 @@
       <c r="G14" s="10" t="n">
         <v>3.5</v>
       </c>
-      <c r="H14" s="7">
+      <c r="H14" s="20">
         <f>IF(F14=0,"",(E14-F14)/F14)</f>
         <v/>
       </c>
-      <c r="I14" s="7">
+      <c r="I14" s="20">
         <f>IF(G14=0,"",(G14-E14)/E14)</f>
         <v/>
       </c>
@@ -3992,7 +4005,7 @@
         <v>4</v>
       </c>
       <c r="E15" s="10" t="n">
-        <v>4</v>
+        <v>4.589</v>
       </c>
       <c r="F15" s="10" t="n">
         <v>3.7</v>
@@ -4000,11 +4013,11 @@
       <c r="G15" s="10" t="n">
         <v>4.4</v>
       </c>
-      <c r="H15" s="7">
+      <c r="H15" s="20">
         <f>IF(F15=0,"",(E15-F15)/F15)</f>
         <v/>
       </c>
-      <c r="I15" s="7">
+      <c r="I15" s="20">
         <f>IF(G15=0,"",(G15-E15)/E15)</f>
         <v/>
       </c>
@@ -4183,17 +4196,17 @@
           <t>极端下跌</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="22" t="n">
         <v>-0.15</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="22" t="n">
         <v>-0.075</v>
       </c>
       <c r="D5" s="5">
         <f>$B$2*C5</f>
         <v/>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="20" t="n">
         <v>-0.115</v>
       </c>
       <c r="F5" s="5">
@@ -4207,17 +4220,17 @@
           <t>继续下跌</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="22" t="n">
         <v>-0.1</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="22" t="n">
         <v>-0.055</v>
       </c>
       <c r="D6" s="5">
         <f>$B$2*C6</f>
         <v/>
       </c>
-      <c r="E6" s="7" t="n">
+      <c r="E6" s="20" t="n">
         <v>-0.08500000000000001</v>
       </c>
       <c r="F6" s="5">
@@ -4231,17 +4244,17 @@
           <t>震荡</t>
         </is>
       </c>
-      <c r="B7" s="17" t="n">
+      <c r="B7" s="22" t="n">
         <v>0.03</v>
       </c>
-      <c r="C7" s="17" t="n">
+      <c r="C7" s="22" t="n">
         <v>0.015</v>
       </c>
       <c r="D7" s="5">
         <f>$B$2*C7</f>
         <v/>
       </c>
-      <c r="E7" s="7" t="n">
+      <c r="E7" s="20" t="n">
         <v>0.025</v>
       </c>
       <c r="F7" s="5">
@@ -4255,17 +4268,17 @@
           <t>超跌反弹</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="22" t="n">
         <v>0.1</v>
       </c>
-      <c r="C8" s="17" t="n">
+      <c r="C8" s="22" t="n">
         <v>0.055</v>
       </c>
       <c r="D8" s="5">
         <f>$B$2*C8</f>
         <v/>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="20" t="n">
         <v>0.08500000000000001</v>
       </c>
       <c r="F8" s="5">
@@ -4279,17 +4292,17 @@
           <t>强势修复</t>
         </is>
       </c>
-      <c r="B9" s="17" t="n">
+      <c r="B9" s="22" t="n">
         <v>0.15</v>
       </c>
-      <c r="C9" s="17" t="n">
+      <c r="C9" s="22" t="n">
         <v>0.08</v>
       </c>
       <c r="D9" s="5">
         <f>$B$2*C9</f>
         <v/>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="20" t="n">
         <v>0.125</v>
       </c>
       <c r="F9" s="5">
@@ -4310,7 +4323,7 @@
           <t>输入大盘涨跌（如 -0.1 表示跌10%）：</t>
         </is>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="23" t="n">
         <v>-0.1</v>
       </c>
     </row>
@@ -4360,7 +4373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A41"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -4373,9 +4386,7 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="15" t="inlineStr">
         <is>
@@ -4418,9 +4429,7 @@
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" t="inlineStr"/>
-    </row>
+    <row r="9"/>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
@@ -4484,9 +4493,7 @@
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr"/>
-    </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
@@ -4522,51 +4529,617 @@
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" t="inlineStr"/>
-    </row>
+    <row r="25"/>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>【重要提醒】</t>
+          <t>【自动更新行情】</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>• 本表仅为投资辅助工具，不构成投资建议</t>
+          <t>1. 安装依赖：pip install -r requirements.txt</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>• 止损价触发后请严格执行，不要抱幻想</t>
+          <t>2. 手动更新：python3 update_portfolio_excel.py</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>• 加仓须满足「每日监控」表底部条件检查</t>
+          <t>3. 每日定时：./run_daily_update.sh（建议交易日 15:30 运行）</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>• 红利ETF和沪深300ETF买入价按估算填入，请以实际成交价更新成本</t>
+          <t>4. 更新内容：现价、涨跌幅、上证指数、跌停家数、更新日志</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr"/>
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>5. Mac/Linux 定时任务示例：</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t xml:space="preserve">   30 15 * * 1-5 cd /path/to/workspace &amp;&amp; ./run_daily_update.sh &gt;&gt; update.log 2&gt;&amp;1</t>
+        </is>
+      </c>
+    </row>
+    <row r="33"/>
+    <row r="34">
+      <c r="A34" s="15" t="inlineStr">
+        <is>
+          <t>【重要提醒】</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>• 本表仅为投资辅助工具，不构成投资建议</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>• 止损价触发后请严格执行，不要抱幻想</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>• 加仓须满足「每日监控」表底部条件检查</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>• 红利ETF和沪深300ETF买入价按估算填入，请以实际成交价更新成本</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>• 非交易时段/周末运行将获取最近一个交易日收盘数据</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>基准日期：2026-07-17  |  账户总市值：434,050 元</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>更新时间</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>代码</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>名称</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>现价</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>涨跌幅%</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>行情日期</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>数据源</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>588810</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>科创芯片ETF</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>2.557</v>
+      </c>
+      <c r="E2" t="n">
+        <v>-8.19</v>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>fund_etf_spot_em</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>159819</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AI智能ETF</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>1.82</v>
+      </c>
+      <c r="E3" t="n">
+        <v>-8.08</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>fund_etf_spot_em</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>002384</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>东山精密</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>241.92</v>
+      </c>
+      <c r="E4" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>stock_zh_a_daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>002475</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>立讯精密</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>58.05</v>
+      </c>
+      <c r="E5" t="n">
+        <v>-5.73</v>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>stock_zh_a_daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>603228</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>景旺电子</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>71.7</v>
+      </c>
+      <c r="E6" t="n">
+        <v>1.29</v>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>stock_zh_a_daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>600183</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>生益科技</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>132.29</v>
+      </c>
+      <c r="E7" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>stock_zh_a_daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>515880</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>通信ETF</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0.659</v>
+      </c>
+      <c r="E8" t="n">
+        <v>-9.970000000000001</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>fund_etf_spot_em</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>600487</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>亨通光电</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="E9" t="n">
+        <v>-9.960000000000001</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>stock_zh_a_daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>001359</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>平安电工</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>96.19</v>
+      </c>
+      <c r="E10" t="n">
+        <v>-10</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>stock_zh_a_daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>002156</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>通富微电</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>68.36</v>
+      </c>
+      <c r="E11" t="n">
+        <v>-9.99</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>stock_zh_a_daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>002222</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>福晶科技</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>60.05</v>
+      </c>
+      <c r="E12" t="n">
+        <v>-8.92</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>stock_zh_a_daily</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>510880</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>红利ETF</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3.135</v>
+      </c>
+      <c r="E13" t="n">
+        <v>-0.35</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>fund_etf_spot_em</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>510300</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>沪深300ETF</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>4.589</v>
+      </c>
+      <c r="E14" t="n">
+        <v>-3.45</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-07-19</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>fund_etf_spot_em</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-19 06:52:31</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>000001</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>上证指数</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3764.155</v>
+      </c>
+      <c r="E15" t="n">
+        <v>-3.05</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>stock_zh_index_daily</t>
         </is>
       </c>
     </row>

</xml_diff>